<commit_message>
feat: add documentation for FastAPI error handling, Pydantic schemas, and dependency injection while updating existing guides
</commit_message>
<xml_diff>
--- a/tests/temp/js.xlsx
+++ b/tests/temp/js.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -476,7 +476,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Що станеться при завантаженні цієї HTML-сторінки в браузері?</t>
+          <t>Що виведе цей код у консоль?</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -486,48 +486,48 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Виведеться вікно alert із повідомленням "Привіт, світ!", а зовнішній файл script.js проігнорується.</t>
+          <t>undefined 0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Завантажиться та виконається зовнішній файл script.js, а вміст всередині тегу (виклик alert) буде проігноровано.</t>
+          <t>null 0</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Обидва скрипти виконаються: спочатку script.js, а потім alert.</t>
+          <t>undefined 1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Виникне синтаксична помилка HTML.</t>
+          <t>TypeError: Cannot read properties of null</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/iqqb9e.png</t>
+          <t>https://files.catbox.moe/zap9sr.png</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Якщо в тегу &lt;script&gt; вказано атрибут src, то будь-який вміст всередині тегу ігнорується. Браузер завантажить і виконає лише зовнішній файл.</t>
+          <t>Опціональний ланцюжок `?.` негайно припиняє обчислення, якщо значення перед ним є `null` або `undefined`. Оскільки `user` дорівнює `null`, обчислення виразу припиняється: метод `name()` не викликається, а вираз `count++` взагалі не виконується. Результатом виразу є `undefined`, а змінна `count` залишається рівною `0`.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Що станеться під час виконання цього коду?</t>
+          <t>Який результат виконання наступного коду?</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -537,22 +537,22 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Спочатку з'явиться вікно "Привіт", а потім по черзі вікна "1" та "2".</t>
+          <t>undefined</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>З'явиться вікно "Привіт", після чого виникне помилка (наприклад, TypeError).</t>
+          <t>Помилка синтаксису (SyntaxError)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Виведеться тільки "1" та "2", а перша інструкція проігнорується.</t>
+          <t>Об'єкт залишиться без змін, помилки не буде</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Код виконається без помилок, але нічого не виведе.</t>
+          <t>"Шевченка"</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -562,23 +562,23 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/v7s3pj.png</t>
+          <t>https://files.catbox.moe/hrigbm.png</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Через відсутність крапки з комою після першого alert, JavaScript не вставиться автоматично перед квадратними дужками. Він трактуватиме це як alert("Привіт")[1, 2].forEach(alert). Оскільки alert повертає undefined, спроба отримати властивість [1, 2] від undefined призведе до помилки.</t>
+          <t>Опціональний ланцюжок `?.` не можна використовувати в лівій частині оператора присвоювання. Конструкція `user?.address?.street = ...` призведе до помилки `SyntaxError: Invalid left-hand side in assignment`, оскільки це по суті спроба присвоїти значення результату обчислення виразу (який може повернути `undefined`), що є недопустимим у JavaScript.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Чи є цей код синтаксично коректним у JavaScript?</t>
+          <t>Що буде виведено в консоль після виконання наступного коду?</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -588,48 +588,48 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Так, це звичайний багаторядковий коментар.</t>
+          <t>true "app"</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ні, вкладені багаторядкові коментарі не підтримуються, тому виникне помилка.</t>
+          <t>false "app"</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Так, але лише якщо увімкнено суворий режим "use strict".</t>
+          <t>true undefined</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Так, але внутрішній коментар буде розцінено як звичайний текст.</t>
+          <t>false undefined</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/uabns2.png</t>
+          <t>https://files.catbox.moe/62fv0l.png</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>У JavaScript вкладені багаторядкові коментарі виду /* ... /* ... */ ... */ не підтримуються. Закриваючий символ */ внутрішнього коментаря закриє весь зовнішній коментар передчасно, що призведе до помилки синтаксису для залишку коду.</t>
+          <t>`Symbol.for("app")` створює або шукає символ у глобальному реєстрі символів. Натомість `Symbol("app")` створює унікальний локальний символ, який не реєструється глобально. Тому `sym1 === sym2` є `false`. Метод `Symbol.keyFor(sym)` шукає ім'я тільки для глобальних символів, зареєстрованих через `Symbol.for`, тому для локального символу `sym2` він повертає `undefined`.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Що станеться при виконанні цього коду?</t>
+          <t>Скільки елементів буде в масивах, виведених у консоль?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -639,22 +639,22 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Код завершиться з помилкою ReferenceError: x is not defined.</t>
+          <t>2 2</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Код успішно виконається і виведе спочатку "Початок роботи", а потім "5".</t>
+          <t>1 0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Виникне помилка SyntaxError: "use strict" must be first.</t>
+          <t>2 0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Директива "use strict" буде проігнорована, оскільки перед нею є інший код (крім коментарів), тому x створиться як глобальна змінна, і код виведе "5".</t>
+          <t>1 1</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -664,23 +664,23 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/6u9p0k.png</t>
+          <t>https://files.catbox.moe/wn4h31.png</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Директива "use strict" має знаходитися на самому початку файлу (дозволяються лише коментарі перед нею). Оскільки перед нею викликається alert(), вона ігнорується, і код виконується в нестрогому режимі. У нестрогому режимі присвоєння неоголошеній змінній x = 5 автоматично створює глобальну змінну, тому помилки не буде.</t>
+          <t>Метод `Object.keys(user)` повертає масив лише рядкових властивостей об'єкта, тому він міститиме лише один елемент (`"name"`). Символьні властивості ігноруються. Метод `Object.getOwnPropertySymbols(user)` повертає масив виключно символьних властивостей об'єкта, тому він також поверне масив з одним елементом (створеним символом `Symbol("age")`).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Який буде результат виконання цього коду?</t>
+          <t>Який результат виконання цього коду?</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -690,99 +690,99 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Виведеться "Світ".</t>
+          <t>undefined true</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Виведеться "Привіт".</t>
+          <t>"data" true</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Помилка: SyntaxError (змінну message вже було оголошено).</t>
+          <t>undefined false</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Виведеться "ПривітСвіт".</t>
+          <t>"data" false</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/2ztoyi.png</t>
+          <t>https://files.catbox.moe/ejjaeq.png</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Оголошення змінної за допомогою let або const з тим самим ім'ям в тій самій області видимості вдруге призводить до помилки SyntaxError.</t>
+          <t>Хоча символьні властивості ігноруються в циклах `for..in` та методі `Object.keys()`, метод `Object.assign()` копіює як рядкові, так і символьні властивості при клонуванні чи об'єднанні об'єктів. Тому `clone` отримає властивість `key`, її значення буде `"data"`, а оператор `in` поверне `true`.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Виберіть усі ПРАВИЛЬНІ (допустимі) імена змінних у JavaScript.</t>
+          <t>Що відбудеться при спробі виконати наступний код?</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Multiple Choice</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>let $ = 10;</t>
+          <t>undefined</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>let _user = "Ivan";</t>
+          <t>"Error"</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>let 2ndPlace = "Silver";</t>
+          <t>"Symbol(test)"</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>let my-variable = 5;</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>let return = true;</t>
-        </is>
-      </c>
+          <t>"test"</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1,2</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>45</v>
-      </c>
-      <c r="J7" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://files.catbox.moe/5ble4l.png</t>
+        </is>
+      </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Імена змінних можуть містити букви, цифри, $ та _, але не можуть починатися з цифри (2ndPlace — неправильно), містити дефіс (my-variable — неправильно) або збігатися з зарезервованими словами (return — зарезервоване слово). Символи $ та _ є допустимими ідентифікаторами.</t>
+          <t>Символи в JavaScript не підлягають автоматичному (неявному) перетворенню на рядок. Спроба додати символ до рядка за допомогою оператора `+` викликає виняток `TypeError: Cannot convert a Symbol value to a string`. У результаті виконується блок `catch`, який виводить у консоль рядок `"Error"`.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Чому для однієї константи використано великі літери (COLOR_RED), а для іншої — маленькі (pageLoadTime)?</t>
+          <t>Яке значення виведеться у консоль після порівняння опису локального та глобального символу?</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -792,22 +792,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>COLOR_RED — це глобальна змінна, а pageLoadTime — локальна.</t>
+          <t>false</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Великі літери використовуються для констант, значення яких відоме до виконання коду (hardcoded), а маленькі — для констант, які обчислюються під час виконання (runtime).</t>
+          <t>true</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Це лише особисте уподобання розробника, технічної різниці немає і правила іменування не відрізняються.</t>
+          <t>TypeError</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Константи з великими літерами не дозволяють змінювати значення, а з маленькими — дозволяють.</t>
+          <t>Помилка, бо keyFor не можна порівнювати з description</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -817,23 +817,23 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/13nc8v.png</t>
+          <t>https://files.catbox.moe/ey0inc.png</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Згідно з практикою розробки, константи у верхньому регістрі (наприклад, COLOR_RED) використовуються для значень, які заздалегідь відомі до початку виконання програми (hardcoded). Для констант, що обчислюються під час виконання (наприклад, pageLoadTime), використовується звичайний верблюжий регістр (camelCase).</t>
+          <t>Властивість `.description` повертає опис символу як рядок (для `localSym` це `"id"`). Метод `Symbol.keyFor(globalSym)` шукає ім'я глобального символу у глобальному реєстрі та повертає його як рядок, що для `Symbol.for("id")` також дорівнює `"id"`. Оскільки обидва вирази повертають однаковий рядок `"id"`, оператор строгого порівняння повертає `true`.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Що відбудеться при спробі запустити цей код?</t>
+          <t>Що виведеться в консоль при серіалізації об'єкта із символьним ключем через JSON.stringify?</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -843,48 +843,48 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Код виведе повідомлення "Я люблю JS" без помилок.</t>
+          <t>null</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Виникне помилка ReferenceError, оскільки змінна message не була оголошена за допомогою let, const або var.</t>
+          <t>"{"tempFormat":"value"}"</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Виникне помилка SyntaxError, тому що рядок "use strict" має містити одинарні лапки.</t>
+          <t>"{}"</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Змінна message автоматично оголоситься як константа.</t>
+          <t>"{"Symbol(temp)":"value"}"</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I9" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/fs7qn6.png</t>
+          <t>https://files.catbox.moe/kbvg21.png</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>У суворому режимі ("use strict") не дозволяється неявне створення змінних без ключових слів let, const або var. Спроба присвоїти значення неоголошеній змінній викликає ReferenceError.</t>
+          <t>Функція `JSON.stringify()` повністю ігнорує будь-які символьні ключі в об'єктах при серіалізації. Оскільки об'єкт `obj` не має інших властивостей, окрім символьного ключа `sym`, результатом серіалізації буде порожній JSON-об'єкт `"{}"`.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Що виведе цей код?</t>
+          <t>Яке значення буде виведено в консоль після додавання об'єкта до числа?</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -894,99 +894,99 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>"string"</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>"number"</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>"object"</t>
+          <t>"105"</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>"null"</t>
+          <t>"205"</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/el8wq9.png</t>
+          <t>https://files.catbox.moe/v6dw1h.png</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>У JavaScript змінні є динамічно типізованими. Спочатку змінній data присвоєно рядок, потім число, а врешті-решт — null. Оператор typeof null повертає "object" через історичну помилку в мові JavaScript, яка залишається незмінною для зворотної сумісності.</t>
+          <t>Оператор бінарного додавання `+` використовує підказку перетворення типу `"default"`. За відсутності методу `Symbol.toPrimitive`, для підказки `"default"` (як і для `"number"`) JavaScript спочатку шукає та викликає метод `valueOf()`. Оскільки `valueOf` існує та повертає число `10`, об'єкт перетворюється на `10`, і вираз `10 + 5` дає результат `15`.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Які значення отримають змінні a, b та c відповідно?</t>
+          <t>Що виведеться в консоль при виконанні наступних операцій над об'єктом, який має лише метод toString?</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Multiple Choice</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>a отримає значення Infinity</t>
+          <t>NaN "102"</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>b отримає значення NaN</t>
+          <t>20 12</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>c отримає значення NaN</t>
+          <t>NaN 12</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>b та c викликають фатальну помилку, яка зупиняє виконання скрипту.</t>
+          <t>20 "102"</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1,2,3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/ws4x5l.png</t>
+          <t>https://files.catbox.moe/rsyrrw.png</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Ділення на нуль 1 / 0 дає Infinity. Множення некоректного рядка на число дає NaN. Оскільки NaN є "причепливим" (sticky), будь-яка подальша математична операція з ним (наприклад, NaN + 5) також повертає NaN. Обчислення в JS є безпечними та не зупиняють програму.</t>
+          <t>Для операції `obj * 2` (підказка `"number"`) та операції `obj + 2` (підказка `"default"`) JavaScript шукає метод `valueOf()`. Оскільки його немає, викликається `toString()`, що повертає рядок `"10"`. При множенні рядок `"10"` перетворюється на число `10` (`10 * 2 = 20`). При додаванні рядок `"10"` додається до числа `2`, що призводить до конкатенації рядків: `"10" + 2 = "102"`.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Що виведе цей код?</t>
+          <t>Який результат роботи наступного коду, де перетворення налаштовано через Symbol.toPrimitive?</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -996,22 +996,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>NaN</t>
+          <t>5 "hellohello"</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>NaN "hello"</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5 "hello"</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>undefined</t>
+          <t>TypeError</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1021,23 +1021,23 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/bkecxn.png</t>
+          <t>https://files.catbox.moe/7qdfe8.png</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>NaN є причепливим значенням і майже в будь-яких математичних операціях повертає NaN. Проте є єдиний виняток: операція піднесення до степеня NaN ** 0 дорівнює 1 (як і будь-яке інше число в степені 0).</t>
+          <t>Унарний плюс `+obj` викликає перетворення типу з підказкою `"number"`, тому `Symbol.toPrimitive` повертає `5`. Додавання об'єкта до рядка `obj + ""` викликає перетворення з підказкою `"default"`, тому метод повертає рядок `"hello"`. В консоль буде виведено `5 "hello"`.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Що виведе цей код?</t>
+          <t>Що виведе цей код у консоль у випадку повернення об'єкта з методу valueOf?</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1047,48 +1047,48 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>NaN</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>TypeError</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Виникне помилка SyntaxError через невідомий символ n.</t>
+          <t>"[object Object]1"</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Виникне помилка TypeError при порівнянні різних типів.</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/vskr1h.png</t>
+          <t>https://files.catbox.moe/86mb9u.png</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Символ n наприкінці цілого числа позначає тип BigInt. typeof value1 поверне "number", а typeof value2 поверне "bigint". Вони не є однаковими, тому порівняння повертає false.</t>
+          <t>Математична операція віднімання `obj - 1` потребує перетворення з підказкою `"number"`. Спочатку викликається `valueOf()`, але він повертає не примітив, а об'єкт `{}`. За історичними правилами JavaScript, якщо метод `valueOf` або `toString` повертає об'єкт, це значення ігнорується, і здійснюється спроба викликати інший метод. Тож викликається `toString()`, що повертає `"3"`, який перетворюється на число `3`, і обчислюється `3 - 1 = 2`.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Що саме буде виведено на екран у вікні alert?</t>
+          <t>Який результат виконання коду, якщо Symbol.toPrimitive повертає об'єкт?</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1098,48 +1098,48 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Привіт, Гість!</t>
+          <t>TypeError</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Привіт, ${user}!</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Привіт, undefined!</t>
+          <t>Помилка не виникне, повернеться undefined</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Привіт, !</t>
+          <t>NaN</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/rtphwy.png</t>
+          <t>https://files.catbox.moe/5sbuw4.png</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Інтерполяція змінних за допомогою ${...} працює ТІЛЬКИ у зворотних лапках (backticks: `...`). У подвійних "..." та одинарних '...' лапках цей запис сприймається як звичайний текст, тому буде виведено дослівно Привіт, ${user}!.</t>
+          <t>На відміну від застарілих методів `toString` та `valueOf`, які при поверненні об'єкта ігноруються, метод `Symbol.toPrimitive` є строгим. Він зобов'язаний повернути примітивне значення. Якщо він повертає об'єкт, JavaScript негайно викликає помилку типу `TypeError: Cannot convert object to primitive value`.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Що виведе цей код та чому?</t>
+          <t>Що виведеться в консоль після порівняння двох об'єктів?</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1149,48 +1149,48 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>"null", оскільки null є окремим типом даних.</t>
+          <t>TypeError</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>"object", тому що null є об'єктом.</t>
+          <t>false</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>"object", і це є офіційно визнаною помилкою в реалізації оператора typeof в JavaScript.</t>
+          <t>true</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>"undefined", оскільки значення не визначено.</t>
+          <t>Порівняння неможливе</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/7sg5ct.png</t>
+          <t>https://files.catbox.moe/e8m3sp.png</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Результатом typeof null є "object". Це відома помилка в мові з її найперших версій, яка зберігається заради сумісності зі старим кодом. Насправді null — це окремий примітивний тип даних, а не об'єкт.</t>
+          <t>Оператори порівняння менше/більше (`&lt;`, `&gt;`) використовують підказку `"number"`. Для `obj1` метод `valueOf` повертає сам об'єкт (дефолтна поведінка), тому викликається `toString()`, що дає `"apple"`. Для `obj2` викликається `valueOf()`, що повертає `100`. Порівняння `"apple" &gt; 100` намагається привести `"apple"` до числа, що дає `NaN`. Будь-яке порівняння з `NaN` завжди повертає `false`.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Який тип даних поверне typeof alert у браузері?</t>
+          <t>Що буде виведено в консоль після запису значення за ключем-об'єктом?</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1200,48 +1200,48 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>"object"</t>
+          <t>42</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>"function"</t>
+          <t>42 або undefined в залежності від браузера</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>"undefined"</t>
+          <t>undefined</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>"string"</t>
+          <t>TypeError</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/7yr7bf.png</t>
+          <t>https://files.catbox.moe/dt3t4f.png</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>alert є вбудованою функцією. Оператор typeof для будь-якої функції повертає рядок "function". Хоча технічно в JavaScript немає окремого типу даних "function" (функції є об'єктами), така поведінка typeof реалізована для зручності.</t>
+          <t>Коли об'єкт використовується як ключ властивості (`container[obj]`), відбувається перетворення з підказкою `"string"`. Викликається метод `toString()`, який повертає рядок `"test"`. Отже, значення `42` записується под ключем `"test"`, і пряме звернення `container["test"]` повертає `42`.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Що буде виведено у вікні alert?</t>
+          <t>Який результат порівняння за допомогою нестрогої рівності (==) в даному коді?</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1251,22 +1251,22 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>NaN, 0</t>
+          <t>true</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0, 0</t>
+          <t>Оскільки типи різні, завжди false</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>NaN, NaN</t>
+          <t>TypeError</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0, NaN</t>
+          <t>false</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -1276,23 +1276,23 @@
         </is>
       </c>
       <c r="I17" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/qy1v7g.png</t>
+          <t>https://files.catbox.moe/eop6pj.png</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>При перетворенні на число за допомогою Number(), значення undefined перетворюється на NaN, а null перетворюється на 0. Це поширена помилка серед новачків, які очікують 0 в обох випадках.</t>
+          <t>Нестрога рівність `obj == 2` використовує підказку `"default"`. За відсутності `Symbol.toPrimitive` та `valueOf`, JavaScript звертається до методу `toString()`, який повертає рядок `"2"`. Після цього порівняння зводиться до `"2" == 2`. Оскільки типи різні, рядок `"2"` приводиться до числа `2`. Обчислюється `2 == 2`, що дає `true`.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Який тип даних матиме змінна result?</t>
+          <t>Що виведеться в консоль при додаванні об'єкта, чий toString повертає число?</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1302,48 +1302,48 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>"string"</t>
+          <t>NaN</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>"number"</t>
+          <t>"500100"</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>"NaN"</t>
+          <t>Помилка через повернення числа з toString</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>"object"</t>
+          <t>600</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I18" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/2abds6.png</t>
+          <t>https://files.catbox.moe/4r2vq4.png</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Математичний оператор ділення / автоматично приводить свої операнди до чисел. Рядки "10" та "2" перетворюються на числа 10 та 2, відповідно ділення дає 5, яке є типом "number".</t>
+          <t>Всупереч назві, метод `toString` не зобов'язаний повертати саме тип рядок, він просто повинен повернути примітив. Тут `toString` повертає число `500`. Оскільки у виразі `user + 100` використовується підказка `"default"` і дефолтний `valueOf` ігнорується, викликається `toString()`. Об'єкт перетворюється на число `500`, і результат додавання `500 + 100` дорівнює `600`.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Що виведе цей код?</t>
+          <t>Що виведеться в консоль при додаванні двох об'єктів?</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1353,99 +1353,99 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>"defaultdefault"</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>NaN</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>NaN</t>
+          <t>"numbernumber"</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>TypeError</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/8529gh.png</t>
+          <t>https://files.catbox.moe/g7060z.png</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>У JavaScript при перетворенні на булевий тип будь-які непусті рядки (включаючи рядок із нулем "0" та рядок із пробілом " ") стають true. Лише абсолютно порожній рядок "" стає false. Таким чином, bool1 та bool2 дорівнюють true, і операція true &amp;&amp; true дає true.</t>
+          <t>Оператор бінарного додавання `+` використовує підказку `"default"`. Обидва операнди є об'єктами, тому метод `[Symbol.toPrimitive]` викликається для кожного з них з аргументом `"default"`, повертаючи рядок `"default"`. Після цього два рядки конкатенуються, даючи `"defaultdefault"`.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Які з цих змінних отримають значення false?</t>
+          <t>Який вбудований об'єкт є винятком і реалізує перетворення з підказкою "default" як для "string", а не як для "number"?</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Checkbox</t>
+          <t>Multiple Choice</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>RegExp</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>Немає винятків, усі працюють однаково</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>Array</t>
         </is>
       </c>
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>1,3,4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/mrcmoj.png</t>
+          <t>https://files.catbox.moe/3vgzu1.png</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Значення, які інтуїтивно є "порожніми" (такі як 0, порожній рядок "", null, undefined та NaN), при булевому перетворенні стають false. Будь-які інші значення (наприклад, непустий рядок "вітаю") перетворюються на true.</t>
+          <t>Всі вбудовані об'єкти в JavaScript (за винятком `Date`) реалізують перетворення для підказки `"default"` так само, як і для `"number"` (повертаючи числове значення або звертаючись до `valueOf`). Об'єкт `Date` є єдиним вбудованим винятком: він реалізує підказку `"default"` як для `"string"`, повертаючи рядкове представлення дати.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Для чого потрібна дана конструкція в JavaScript розробці?</t>
+          <t>Що виведе цей код у консоль?</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1455,41 +1455,41 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Вона створює новий об'єкт та додає до нього метод alert.</t>
+          <t>TypeError</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Це спосіб безпечно активувати суворий режим "use strict" лише для конкретного блоку коду (функції-обгортки), не впливаючи на інший код.</t>
+          <t>NaN</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Вона використовується для оптимізації роботи з кешем браузера.</t>
+          <t>"105"</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Це обов'язковий синтаксис для підключення зовнішніх файлів скриптів.</t>
+          <t>15</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://files.catbox.moe/b64tnk.png</t>
+          <t>https://files.catbox.moe/bk39c7.png</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Директиву 'use strict' можна вказувати на початку окремої функції, щоб увімкнути суворий режим лише для коду всередині неї. Функція-обгортка (function() { ... })() негайно викликається і локалізує строгий режим, що корисно при об'єднанні декількох скриптів (наприклад, у старіших версіях браузерів, де консоль не підтримує strict mode глобально).</t>
+          <t>Унарний плюс `+obj` викликає перетворення об'єкта з підказкою `"number"`. Викликається `valueOf()`, що повертає примітив-рядок `"10"`. Після цього унарний плюс перетворює отриманий рядок `"10"` на число `10`. Далі до результату додається `5`, отримуючи `10 + 5 = 15`.</t>
         </is>
       </c>
     </row>

</xml_diff>